<commit_message>
Add house import/export functionality, excel samples, and UI updates
</commit_message>
<xml_diff>
--- a/public/sample_material_import.xlsx
+++ b/public/sample_material_import.xlsx
@@ -124,7 +124,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -134,13 +134,28 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F9B3A"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -155,8 +170,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,45 +479,45 @@
   <cols>
     <col min="1" max="1" width="34.135" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="15.139" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="12.854" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="34.135" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" customHeight="1" ht="26">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>